<commit_message>
Update Test Cases, Bug Reports and formatting
</commit_message>
<xml_diff>
--- a/Bug_Reports/TickTick_Bug_Reports.xlsx
+++ b/Bug_Reports/TickTick_Bug_Reports.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQA\Intern\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQA\Intern\innovaxel-sqa-assessment-ticktick\Bug_Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84E202D1-1649-47C4-9CE1-36B4CC4B515C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5604F08-C125-42CA-821C-D170C3D8907E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="59">
   <si>
     <t>Expected Result</t>
   </si>
@@ -52,9 +52,6 @@
     <t>No Delete Option for Habits</t>
   </si>
   <si>
-    <t>1. Go to Habit tab 2. Create a habit 3. Try to delete it</t>
-  </si>
-  <si>
     <t>User should be able to delete unwanted habits</t>
   </si>
   <si>
@@ -64,9 +61,6 @@
     <t>Medium</t>
   </si>
   <si>
-    <t>Yes</t>
-  </si>
-  <si>
     <t>Add delete or archive functionality for habits</t>
   </si>
   <si>
@@ -76,9 +70,6 @@
     <t>Task Can Be Saved Without Title</t>
   </si>
   <si>
-    <t>1. Tap + button 2. Enter only description 3. Tap save</t>
-  </si>
-  <si>
     <t>App should require a task title</t>
   </si>
   <si>
@@ -97,9 +88,6 @@
     <t>Unclear Bottom Navigation Icons</t>
   </si>
   <si>
-    <t>1. Open the app 2. Look at bottom tab icons</t>
-  </si>
-  <si>
     <t>Icons should be clear and self-explanatory</t>
   </si>
   <si>
@@ -115,9 +103,6 @@
     <t>No Confirmation Dialog on Task Deletion</t>
   </si>
   <si>
-    <t>1. Long press a task 2. Select Delete</t>
-  </si>
-  <si>
     <t>App should show confirmation warning before permanent deletion</t>
   </si>
   <si>
@@ -133,9 +118,6 @@
     <t>Poor Search &amp; Filter Usability</t>
   </si>
   <si>
-    <t>1. Go to Search tab 2. Try using search and filters</t>
-  </si>
-  <si>
     <t>Search should be simple and filters well organized</t>
   </si>
   <si>
@@ -151,9 +133,6 @@
     <t>Duplicate Tasks Allowed with Same Name &amp; Date</t>
   </si>
   <si>
-    <t>1. Create task with title + due date 2. Create another identical task</t>
-  </si>
-  <si>
     <t>App should prevent or warn about duplicate tasks</t>
   </si>
   <si>
@@ -169,9 +148,6 @@
     <t>Past Due Dates Allowed for New Tasks</t>
   </si>
   <si>
-    <t>1. Create new task 2. Set due date in the past 3. Save</t>
-  </si>
-  <si>
     <t>App should prevent past dates or give clear warning</t>
   </si>
   <si>
@@ -179,13 +155,65 @@
   </si>
   <si>
     <t>Restrict past dates during task creation</t>
+  </si>
+  <si>
+    <t>1. Go to Habit tab 
+2. Create a habit 
+3. Try to delete it</t>
+  </si>
+  <si>
+    <t>1. Tap + button 
+2. Enter only description 
+3. Tap save</t>
+  </si>
+  <si>
+    <t>1. Open the app 
+2. Look at bottom tab icons</t>
+  </si>
+  <si>
+    <t>1. Long press a task 
+2. Select Delete</t>
+  </si>
+  <si>
+    <t>1. Go to Search tab 
+2. Try using search and filters</t>
+  </si>
+  <si>
+    <t>1. Create task with title + due date 
+2. Create another identical task</t>
+  </si>
+  <si>
+    <t>1. Create new task 
+2. Set due date in the past 
+3. Save</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/13sIKH7-TCCuDvxYipXob9jJwWjn79xwb/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1jcW7odK8EJgio9fmXDBwut8oP0x1rvCf/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1Zw7bW565Tu9ZhpxVf2jfX7vpwyB43kvq/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1NMFJp8M4Fd38wU3c-yocCJsp4bAIsAnM/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1oKQZVERn-jiSrW7_GNo-W1x5wRa9Xwi0/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1JKJc108ZgZZP9hFAGjmZlES5Bt4RsiPq/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1hsu5wa1HeZ_DqF4_DUDBowyjNLziDin5/view?usp=drive_link</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -193,6 +221,12 @@
     <font>
       <b/>
       <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -204,7 +238,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -212,23 +246,43 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -574,215 +628,224 @@
     <col min="8" max="8" width="21.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="3" t="s">
+    </row>
+    <row r="3" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="C3" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>19</v>
+      </c>
     </row>
-    <row r="3" spans="1:8" ht="72" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="3" t="s">
+    <row r="4" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>22</v>
+      <c r="G5" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="72" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>28</v>
+    <row r="6" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>34</v>
+    <row r="7" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>39</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" s="3" t="s">
+    <row r="8" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="B8" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="C8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="E8" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="F8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="H8" s="2" t="s">
         <v>44</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>47</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F8" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>52</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G2" r:id="rId1" xr:uid="{32FE19E4-1B8C-4400-B273-94E32E3B8B32}"/>
+    <hyperlink ref="G3" r:id="rId2" xr:uid="{ADE857D9-DEAA-40C5-AF8F-6EC94F7D6E4B}"/>
+    <hyperlink ref="G4" r:id="rId3" xr:uid="{DE6D0ADB-FEEB-49F1-A212-D41B34814769}"/>
+    <hyperlink ref="G5" r:id="rId4" xr:uid="{33188F24-5248-4ACE-B9DD-93A1395FBA87}"/>
+    <hyperlink ref="G6" r:id="rId5" xr:uid="{D0CEBB30-89FD-4484-A393-3E01B44B16E3}"/>
+    <hyperlink ref="G7" r:id="rId6" xr:uid="{8F19D7D3-DE1E-4983-9CE7-78D7B9AD34BF}"/>
+    <hyperlink ref="G8" r:id="rId7" xr:uid="{1EFC066B-D7B9-4673-A7F7-04A7626E2831}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>